<commit_message>
Fixes so TeamsGlobalScoring works with Robi
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionBook/TeamsGlobalScoring-A4.xlsx
+++ b/owlcms/src/main/resources/templates/competitionBook/TeamsGlobalScoring-A4.xlsx
@@ -1,27 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\competitionBook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C7CBAD6-8DA3-4041-AE28-C27D66F3EFCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{83250258-8CB7-4BA0-8C7A-7DDB9BFEE57D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="447" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="447" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Men" sheetId="33" r:id="rId1"/>
     <sheet name="Men Summary" sheetId="44" r:id="rId2"/>
     <sheet name="Women" sheetId="34" r:id="rId3"/>
     <sheet name="Women Summary" sheetId="45" r:id="rId4"/>
+    <sheet name="Mixed" sheetId="46" r:id="rId5"/>
+    <sheet name="Mixed Summary" sheetId="47" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId5"/>
-    <pivotCache cacheId="1" r:id="rId6"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
+    <pivotCache cacheId="1" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="43">
   <si>
     <t>${l.lastName}</t>
   </si>
@@ -164,6 +166,9 @@
   </si>
   <si>
     <t>${competition.womenBestNElseDefault}</t>
+  </si>
+  <si>
+    <t>&lt;jx:forEach items="${mwTeamBest}" var="l" varStatus="lifterLoop"&gt;</t>
   </si>
 </sst>
 </file>
@@ -681,6 +686,51 @@
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0CD45426-5B0A-4FA4-8970-717B67B9CE2D}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="2">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of ${t.get(&quot;Results.PointsScored&quot;)}" fld="0" baseField="1" baseItem="0" numFmtId="2"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FF7C724B-5A3F-4AED-A19C-93B794FCFEA0}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField dataField="1" showAll="0"/>
@@ -1546,4 +1596,247 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7EBA30E-30CE-4620-9A30-11969EFEE9A6}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:S9"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" customWidth="1"/>
+    <col min="8" max="9" width="11.42578125" hidden="1" customWidth="1"/>
+    <col min="10" max="11" width="11.42578125" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="44.140625" style="1" customWidth="1"/>
+    <col min="15" max="19" width="11.42578125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="3.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="N1" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="R1"/>
+      <c r="S1"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2"/>
+      <c r="P2"/>
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="M3" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="R3"/>
+      <c r="S3"/>
+    </row>
+    <row r="4" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="M4"/>
+      <c r="N4"/>
+      <c r="R4"/>
+      <c r="S4"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A5" s="4"/>
+      <c r="B5" s="5" t="str">
+        <f ca="1">IF(A5&gt;0,SUMIF(OFFSET($A$3,0,0,$C$6,1),A5,OFFSET($A$3,0,9,$C$6,1)),"")</f>
+        <v/>
+      </c>
+      <c r="C5" s="4" t="str">
+        <f ca="1">IF(A5&gt;0,RANK(B5,OFFSET(#REF!,0,0,#REF!,2)),"")</f>
+        <v/>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.55118110236220474" bottom="0.43307086614173229" header="0.23622047244094491" footer="0.15748031496062992"/>
+  <pageSetup paperSize="9" scale="76" firstPageNumber="0" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <headerFooter alignWithMargins="0">
+    <oddHeader>&amp;L&amp;14Classement Sinclair - Sinclair Ranking&amp;R&amp;14Hommes - Men</oddHeader>
+    <oddFooter>&amp;R&amp;P</oddFooter>
+  </headerFooter>
+  <colBreaks count="1" manualBreakCount="1">
+    <brk id="19" max="1048575" man="1"/>
+  </colBreaks>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA5FE0B6-555F-4CA2-A4C4-5B7087C35C48}">
+  <dimension ref="A3:B6"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="46.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="19"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="19">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix for mixed teams
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionBook/TeamsGlobalScoring-A4.xlsx
+++ b/owlcms/src/main/resources/templates/competitionBook/TeamsGlobalScoring-A4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\competitionBook\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\local\templates\competitionBook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{83250258-8CB7-4BA0-8C7A-7DDB9BFEE57D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE0FBD4B-CF46-4637-963E-634A500B785F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="447" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="447" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Men" sheetId="33" r:id="rId1"/>
@@ -24,6 +24,7 @@
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId7"/>
     <pivotCache cacheId="1" r:id="rId8"/>
+    <pivotCache cacheId="23" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="46">
   <si>
     <t>${l.lastName}</t>
   </si>
@@ -169,6 +170,15 @@
   </si>
   <si>
     <t>&lt;jx:forEach items="${mwTeamBest}" var="l" varStatus="lifterLoop"&gt;</t>
+  </si>
+  <si>
+    <t>$[if(D3="M",if(C8&lt;&gt;"",if(L3&lt;=C8,K3,0),if(L3&gt;0,K3,0)),if(C9&lt;&gt;"",if(L3&lt;=C9,K3,0),if(L3&gt;0,K3,0)))]</t>
+  </si>
+  <si>
+    <t>${nbWomen+nbMen}</t>
+  </si>
+  <si>
+    <t>$[concatenate(A3)]</t>
   </si>
 </sst>
 </file>
@@ -226,7 +236,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -257,8 +267,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -354,6 +370,28 @@
       <top style="medium">
         <color indexed="8"/>
       </top>
+      <bottom style="medium">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="8"/>
+      </right>
+      <top style="medium">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="8"/>
+      </right>
+      <top/>
       <bottom style="medium">
         <color indexed="8"/>
       </bottom>
@@ -373,7 +411,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -418,6 +456,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Emphase 1" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -514,7 +555,31 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jean-François Lamy" refreshedDate="45781.74989525463" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="8" xr:uid="{AE52AADC-027E-46DB-AB1B-CA969DB382F6}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jean-François Lamy" refreshedDate="46068.565165856482" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="9" xr:uid="{1ACD3D99-8DE1-45FC-B01A-43090277884E}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="M1:N1048576" sheet="Women"/>
+  </cacheSource>
+  <cacheFields count="2">
+    <cacheField name="${t.get(&quot;Results.PointsScored&quot;)}" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="TeamWithSuffix" numFmtId="0">
+      <sharedItems containsBlank="1" count="2">
+        <m/>
+        <s v="$[concatenate(A3,&quot; &quot;,CHAR(quotient(L3-1,C9)+1+64))]"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jean-François Lamy" refreshedDate="46068.565166087959" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="8" xr:uid="{AE52AADC-027E-46DB-AB1B-CA969DB382F6}">
   <cacheSource type="worksheet">
     <worksheetSource ref="M1:N1048576" sheet="Men"/>
   </cacheSource>
@@ -537,10 +602,10 @@
 </pivotCacheDefinition>
 </file>
 
-<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jean-François Lamy" refreshedDate="45781.75348900463" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="9" xr:uid="{1ACD3D99-8DE1-45FC-B01A-43090277884E}">
+<file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jean-François Lamy" refreshedDate="46068.622174074073" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="9" xr:uid="{8E9A4A43-659F-482F-90FA-0BE1F9769341}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="M1:N1048576" sheet="Women"/>
+    <worksheetSource ref="M1:N1048576" sheet="Mixed"/>
   </cacheSource>
   <cacheFields count="2">
     <cacheField name="${t.get(&quot;Results.PointsScored&quot;)}" numFmtId="0">
@@ -549,7 +614,7 @@
     <cacheField name="TeamWithSuffix" numFmtId="0">
       <sharedItems containsBlank="1" count="2">
         <m/>
-        <s v="$[concatenate(A3,&quot; &quot;,CHAR(quotient(L3-1,C9)+1+64))]"/>
+        <s v="$[concatenate(A3)]"/>
       </sharedItems>
     </cacheField>
   </cacheFields>
@@ -562,14 +627,18 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="8">
-  <r>
-    <m/>
-    <x v="0"/>
-  </r>
-  <r>
-    <s v="$[if(D3=&quot;M&quot;,if(C17&lt;&gt;&quot;&quot;,if(L3&lt;=C17,K3,0),if(L3&gt;0,K3,0)),if(C18&lt;&gt;&quot;&quot;,if(L3&lt;=C18,K3,0),if(L3&gt;0,K3,0)))]"/>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="9">
+  <r>
+    <m/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="$[if(D3=&quot;M&quot;,if(C8&lt;&gt;&quot;&quot;,if(L3&lt;=C8,K3,0),if(L3&gt;0,K3,0)),if(C9&lt;&gt;&quot;&quot;,if(L3&lt;=C9,K3,0),if(L3&gt;0,K3,0)))]"/>
     <x v="1"/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
   </r>
   <r>
     <m/>
@@ -599,6 +668,43 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="8">
+  <r>
+    <m/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="$[if(D3=&quot;M&quot;,if(C8&lt;&gt;&quot;&quot;,if(L3&lt;=C8,K3,0),if(L3&gt;0,K3,0)),if(C9&lt;&gt;&quot;&quot;,if(L3&lt;=C9,K3,0),if(L3&gt;0,K3,0)))]"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="9">
   <r>
     <m/>
@@ -640,7 +746,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D43290F7-FE12-4168-9B39-E888C0864416}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D43290F7-FE12-4168-9B39-E888C0864416}" name="PivotTable5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
   <location ref="A1:B4" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField dataField="1" showAll="0"/>
@@ -685,13 +791,13 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0CD45426-5B0A-4FA4-8970-717B67B9CE2D}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0CD45426-5B0A-4FA4-8970-717B67B9CE2D}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField dataField="1" showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="3">
-        <item x="1"/>
+        <item n="$[concatenate(A3,&quot; &quot;,CHAR(quotient(L3-1,C9)+1+64))]" x="1"/>
         <item x="0"/>
         <item t="default"/>
       </items>
@@ -730,14 +836,14 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FF7C724B-5A3F-4AED-A19C-93B794FCFEA0}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{22CB41D1-8607-4634-AD64-A1E0BC38975D}" name="PivotTable1" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField dataField="1" showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="3">
+        <item x="0"/>
         <item x="1"/>
-        <item x="0"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -1236,7 +1342,7 @@
         <v>30</v>
       </c>
       <c r="M3" s="13" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N3" s="13" t="s">
         <v>33</v>
@@ -1475,7 +1581,7 @@
         <v>30</v>
       </c>
       <c r="M3" s="13" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N3" s="13" t="s">
         <v>34</v>
@@ -1594,6 +1700,7 @@
       </c>
     </row>
   </sheetData>
+  <dataConsolidate/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1603,7 +1710,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.42578125" customWidth="1"/>
@@ -1617,12 +1724,12 @@
     <col min="10" max="11" width="11.42578125" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
     <col min="13" max="13" width="11.42578125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="44.140625" style="1" customWidth="1"/>
-    <col min="15" max="19" width="11.42578125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="3.5703125" customWidth="1"/>
+    <col min="14" max="14" width="26.28515625" style="1" customWidth="1"/>
+    <col min="15" max="18" width="11.42578125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="3.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>22</v>
       </c>
@@ -1665,22 +1772,21 @@
       <c r="N1" s="15" t="s">
         <v>31</v>
       </c>
+      <c r="Q1"/>
       <c r="R1"/>
-      <c r="S1"/>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>42</v>
       </c>
-      <c r="M2"/>
+      <c r="M2" s="20"/>
       <c r="N2"/>
       <c r="O2"/>
       <c r="P2"/>
       <c r="Q2"/>
       <c r="R2"/>
-      <c r="S2"/>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
         <v>3</v>
       </c>
@@ -1697,7 +1803,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>27</v>
@@ -1721,21 +1827,21 @@
         <v>32</v>
       </c>
       <c r="N3" s="13" t="s">
-        <v>34</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="Q3"/>
       <c r="R3"/>
-      <c r="S3"/>
-    </row>
-    <row r="4" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="M4"/>
+      <c r="M4" s="21"/>
       <c r="N4"/>
+      <c r="Q4"/>
       <c r="R4"/>
-      <c r="S4"/>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="4"/>
       <c r="B5" s="5" t="str">
         <f ca="1">IF(A5&gt;0,SUMIF(OFFSET($A$3,0,0,$C$6,1),A5,OFFSET($A$3,0,9,$C$6,1)),"")</f>
@@ -1757,15 +1863,15 @@
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -1774,13 +1880,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>41</v>
-      </c>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="C9" s="22"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
@@ -1792,43 +1893,44 @@
     <oddFooter>&amp;R&amp;P</oddFooter>
   </headerFooter>
   <colBreaks count="1" manualBreakCount="1">
-    <brk id="19" max="1048575" man="1"/>
+    <brk id="18" max="1048575" man="1"/>
   </colBreaks>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA5FE0B6-555F-4CA2-A4C4-5B7087C35C48}">
-  <dimension ref="A3:B6"/>
+  <dimension ref="A3:D6"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="46.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="37.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="17" t="s">
         <v>35</v>
       </c>
       <c r="B3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="19">
+        <v>36</v>
+      </c>
+      <c r="B4" s="19"/>
+      <c r="D4" s="18"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="19">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="19"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="18" t="s">
         <v>37</v>
       </c>

</xml_diff>